<commit_message>
Changed to only include v6b, now the good graphs disappeared
</commit_message>
<xml_diff>
--- a/Old version with correct plots/Output/LE_for_mean_age.xlsx
+++ b/Old version with correct plots/Output/LE_for_mean_age.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D133"/>
+  <dimension ref="A1:D123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1644,14 +1644,14 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>North Macedonia</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D77" t="n">
-        <v>44.96972615384617</v>
+        <v>36.45157209230767</v>
       </c>
     </row>
     <row r="78">
@@ -1660,14 +1660,14 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Montenegro</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D78" t="n">
-        <v>44.37803946666668</v>
+        <v>38.56075838461537</v>
       </c>
     </row>
     <row r="79">
@@ -1676,14 +1676,14 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>North Macedonia</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D79" t="n">
-        <v>36.45157209230767</v>
+        <v>42.84707649230774</v>
       </c>
     </row>
     <row r="80">
@@ -1692,14 +1692,14 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Montenegro</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D80" t="n">
-        <v>38.56075838461537</v>
+        <v>35.60673846153851</v>
       </c>
     </row>
     <row r="81">
@@ -1708,14 +1708,14 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D81" t="n">
-        <v>42.84707649230774</v>
+        <v>41.61694615384616</v>
       </c>
     </row>
     <row r="82">
@@ -1724,14 +1724,14 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D82" t="n">
-        <v>35.60673846153851</v>
+        <v>41.59607692307691</v>
       </c>
     </row>
     <row r="83">
@@ -1740,14 +1740,14 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D83" t="n">
-        <v>41.61694615384616</v>
+        <v>33.41685927179487</v>
       </c>
     </row>
     <row r="84">
@@ -1756,94 +1756,94 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Tajikistan</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="D84" t="n">
-        <v>47.93721133333336</v>
+        <v>42.4936580769231</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Turkmenistan</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D85" t="n">
-        <v>42.89285279999998</v>
+        <v>39.41631495384617</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D86" t="n">
-        <v>41.59607692307691</v>
+        <v>41.51013076923078</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="C87" t="n">
         <v>46</v>
       </c>
       <c r="D87" t="n">
-        <v>33.41685927179487</v>
+        <v>35.19236204615387</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Croatia</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D88" t="n">
-        <v>42.4936580769231</v>
+        <v>36.48429895384616</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>2040</v>
+        <v>2050</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Uzbekistan</t>
+          <t>Cyprus</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D89" t="n">
-        <v>46.13572115384613</v>
+        <v>40.77305384615388</v>
       </c>
     </row>
     <row r="90">
@@ -1852,14 +1852,14 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D90" t="n">
-        <v>39.41631495384617</v>
+        <v>41.99678073846154</v>
       </c>
     </row>
     <row r="91">
@@ -1868,14 +1868,14 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D91" t="n">
-        <v>41.51013076923078</v>
+        <v>37.19652516923077</v>
       </c>
     </row>
     <row r="92">
@@ -1884,14 +1884,14 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="C92" t="n">
         <v>46</v>
       </c>
       <c r="D92" t="n">
-        <v>35.19236204615387</v>
+        <v>40.29040667692309</v>
       </c>
     </row>
     <row r="93">
@@ -1900,14 +1900,14 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Croatia</t>
+          <t>France</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D93" t="n">
-        <v>36.48429895384616</v>
+        <v>43.55603929230769</v>
       </c>
     </row>
     <row r="94">
@@ -1916,14 +1916,14 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Cyprus</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D94" t="n">
-        <v>40.77305384615388</v>
+        <v>39.89076156923076</v>
       </c>
     </row>
     <row r="95">
@@ -1932,14 +1932,14 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="D95" t="n">
-        <v>41.99678073846154</v>
+        <v>38.28824529230772</v>
       </c>
     </row>
     <row r="96">
@@ -1948,14 +1948,14 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D96" t="n">
-        <v>37.19652516923077</v>
+        <v>38.13516960000001</v>
       </c>
     </row>
     <row r="97">
@@ -1964,14 +1964,14 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D97" t="n">
-        <v>40.29040667692309</v>
+        <v>43.56531372307696</v>
       </c>
     </row>
     <row r="98">
@@ -1980,14 +1980,14 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D98" t="n">
-        <v>43.55603929230769</v>
+        <v>37.74957692307692</v>
       </c>
     </row>
     <row r="99">
@@ -1996,14 +1996,14 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="C99" t="n">
         <v>46</v>
       </c>
       <c r="D99" t="n">
-        <v>39.89076156923076</v>
+        <v>35.83894175384618</v>
       </c>
     </row>
     <row r="100">
@@ -2012,14 +2012,14 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D100" t="n">
-        <v>38.28824529230772</v>
+        <v>34.98152553846155</v>
       </c>
     </row>
     <row r="101">
@@ -2028,14 +2028,14 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="C101" t="n">
         <v>44</v>
       </c>
       <c r="D101" t="n">
-        <v>38.13516960000001</v>
+        <v>42.27636843076923</v>
       </c>
     </row>
     <row r="102">
@@ -2044,14 +2044,14 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Malta</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D102" t="n">
-        <v>43.56531372307696</v>
+        <v>38.59699417435898</v>
       </c>
     </row>
     <row r="103">
@@ -2060,14 +2060,14 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D103" t="n">
-        <v>37.74957692307692</v>
+        <v>41.30451538461536</v>
       </c>
     </row>
     <row r="104">
@@ -2076,14 +2076,14 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D104" t="n">
-        <v>35.83894175384618</v>
+        <v>36.13842658461541</v>
       </c>
     </row>
     <row r="105">
@@ -2092,14 +2092,14 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C105" t="n">
         <v>47</v>
       </c>
       <c r="D105" t="n">
-        <v>34.98152553846155</v>
+        <v>40.02258055384615</v>
       </c>
     </row>
     <row r="106">
@@ -2108,14 +2108,14 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D106" t="n">
-        <v>42.27636843076923</v>
+        <v>36.37005384615388</v>
       </c>
     </row>
     <row r="107">
@@ -2124,14 +2124,14 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Malta</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D107" t="n">
-        <v>38.59699417435898</v>
+        <v>38.79627003076924</v>
       </c>
     </row>
     <row r="108">
@@ -2140,14 +2140,14 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D108" t="n">
-        <v>41.30451538461536</v>
+        <v>38.84970203076924</v>
       </c>
     </row>
     <row r="109">
@@ -2156,14 +2156,14 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D109" t="n">
-        <v>36.13842658461541</v>
+        <v>43.03918864615384</v>
       </c>
     </row>
     <row r="110">
@@ -2172,14 +2172,14 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Albania</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D110" t="n">
-        <v>40.02258055384615</v>
+        <v>36.94960972307692</v>
       </c>
     </row>
     <row r="111">
@@ -2188,14 +2188,14 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Armenia</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D111" t="n">
-        <v>36.37005384615388</v>
+        <v>38.00919969230771</v>
       </c>
     </row>
     <row r="112">
@@ -2204,14 +2204,14 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Azerbaijan</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="D112" t="n">
-        <v>38.79627003076924</v>
+        <v>39.69467948717951</v>
       </c>
     </row>
     <row r="113">
@@ -2220,14 +2220,14 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Belarus</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D113" t="n">
-        <v>38.84970203076924</v>
+        <v>34.49666342051281</v>
       </c>
     </row>
     <row r="114">
@@ -2236,14 +2236,14 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D114" t="n">
-        <v>43.03918864615384</v>
+        <v>38.92324000000003</v>
       </c>
     </row>
     <row r="115">
@@ -2252,14 +2252,14 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Albania</t>
+          <t>Iceland</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D115" t="n">
-        <v>36.94960972307692</v>
+        <v>42.44716741538461</v>
       </c>
     </row>
     <row r="116">
@@ -2268,14 +2268,14 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Armenia</t>
+          <t>North Macedonia</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D116" t="n">
-        <v>38.00919969230771</v>
+        <v>36.79599230769229</v>
       </c>
     </row>
     <row r="117">
@@ -2284,14 +2284,14 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Azerbaijan</t>
+          <t>Montenegro</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D117" t="n">
-        <v>39.69467948717951</v>
+        <v>38.11075846153849</v>
       </c>
     </row>
     <row r="118">
@@ -2300,14 +2300,14 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Belarus</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D118" t="n">
-        <v>34.49666342051281</v>
+        <v>42.01364615384612</v>
       </c>
     </row>
     <row r="119">
@@ -2316,14 +2316,14 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D119" t="n">
-        <v>38.92324000000003</v>
+        <v>36.1585232820513</v>
       </c>
     </row>
     <row r="120">
@@ -2332,14 +2332,14 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Iceland</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D120" t="n">
-        <v>42.44716741538461</v>
+        <v>41.73692593333336</v>
       </c>
     </row>
     <row r="121">
@@ -2348,14 +2348,14 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="D121" t="n">
-        <v>45.27346222051284</v>
+        <v>40.08008654358976</v>
       </c>
     </row>
     <row r="122">
@@ -2364,14 +2364,14 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="D122" t="n">
-        <v>44.65143963076926</v>
+        <v>32.91865673846157</v>
       </c>
     </row>
     <row r="123">
@@ -2380,174 +2380,14 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>North Macedonia</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D123" t="n">
-        <v>36.79599230769229</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="n">
-        <v>2050</v>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>Montenegro</t>
-        </is>
-      </c>
-      <c r="C124" t="n">
-        <v>44</v>
-      </c>
-      <c r="D124" t="n">
-        <v>38.11075846153849</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="n">
-        <v>2050</v>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>Norway</t>
-        </is>
-      </c>
-      <c r="C125" t="n">
-        <v>45</v>
-      </c>
-      <c r="D125" t="n">
-        <v>42.01364615384612</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="n">
-        <v>2050</v>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Serbia</t>
-        </is>
-      </c>
-      <c r="C126" t="n">
-        <v>46</v>
-      </c>
-      <c r="D126" t="n">
-        <v>36.1585232820513</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="n">
-        <v>2050</v>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>Switzerland</t>
-        </is>
-      </c>
-      <c r="C127" t="n">
-        <v>46</v>
-      </c>
-      <c r="D127" t="n">
-        <v>41.73692593333336</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="n">
-        <v>2050</v>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>Tajikistan</t>
-        </is>
-      </c>
-      <c r="C128" t="n">
-        <v>30</v>
-      </c>
-      <c r="D128" t="n">
-        <v>46.91425961538464</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="n">
-        <v>2050</v>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>Turkmenistan</t>
-        </is>
-      </c>
-      <c r="C129" t="n">
-        <v>34</v>
-      </c>
-      <c r="D129" t="n">
-        <v>41.70118166153842</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="n">
-        <v>2050</v>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>Turkey</t>
-        </is>
-      </c>
-      <c r="C130" t="n">
-        <v>43</v>
-      </c>
-      <c r="D130" t="n">
-        <v>40.08008654358976</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="n">
-        <v>2050</v>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>Ukraine</t>
-        </is>
-      </c>
-      <c r="C131" t="n">
-        <v>48</v>
-      </c>
-      <c r="D131" t="n">
-        <v>32.91865673846157</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="n">
-        <v>2050</v>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="C132" t="n">
-        <v>43</v>
-      </c>
-      <c r="D132" t="n">
         <v>42.72015044102561</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="n">
-        <v>2050</v>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>Uzbekistan</t>
-        </is>
-      </c>
-      <c r="C133" t="n">
-        <v>31</v>
-      </c>
-      <c r="D133" t="n">
-        <v>46.2452164923077</v>
       </c>
     </row>
   </sheetData>

</xml_diff>